<commit_message>
First set of results of the OOP design but time is not handled correctly
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster-backend\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACFC551-8B30-4FBB-9899-8654D3004F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C1DF188-3788-48DC-9AE8-36B4D6CB12E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14070" yWindow="-21720" windowWidth="51840" windowHeight="21240" tabRatio="685" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -646,7 +646,7 @@
         <v>59</v>
       </c>
       <c r="C2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="D2">
         <v>58</v>
@@ -655,7 +655,7 @@
         <v>59</v>
       </c>
       <c r="F2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="G2">
         <v>58</v>
@@ -664,7 +664,7 @@
         <v>59</v>
       </c>
       <c r="I2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First set of promising results after OOP refactoring
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2494B22A-FD0A-4655-BB02-2183BD7346FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC0F6E6-422C-43A0-A53D-E9E07682453B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -640,31 +640,31 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="D2">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="G2">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -699,7 +699,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -708,7 +708,7 @@
         <v>15</v>
       </c>
       <c r="E2">
-        <v>60</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -716,7 +716,7 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -725,7 +725,7 @@
         <v>15</v>
       </c>
       <c r="E3">
-        <v>60</v>
+        <v>60.2</v>
       </c>
     </row>
   </sheetData>
@@ -807,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>57</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -818,13 +818,13 @@
         <v>20000</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -839,7 +839,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>57</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -850,13 +850,13 @@
         <v>20000</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <v>57</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -882,13 +882,13 @@
         <v>20000</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -903,7 +903,7 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>57</v>
+        <v>58.2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -914,13 +914,13 @@
         <v>20000</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -935,7 +935,7 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -946,13 +946,13 @@
         <v>20000</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -967,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>57</v>
+        <v>58.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved reporting, balance tracking
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC0F6E6-422C-43A0-A53D-E9E07682453B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A7AA61-DDC2-4410-B32D-A1BCD5E194E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>

</xml_diff>

<commit_message>
Added cash flow incentives. Added max quantities.
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A7AA61-DDC2-4410-B32D-A1BCD5E194E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F239D22-8A54-415E-9A42-459279C0C526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
   <si>
     <t>name</t>
   </si>
@@ -132,6 +132,33 @@
   </si>
   <si>
     <t>SP6</t>
+  </si>
+  <si>
+    <t>cost_preplan</t>
+  </si>
+  <si>
+    <t>cost_period_1</t>
+  </si>
+  <si>
+    <t>cost_period_2</t>
+  </si>
+  <si>
+    <t>cash_preplan</t>
+  </si>
+  <si>
+    <t>cash_period_1</t>
+  </si>
+  <si>
+    <t>cash_period_2</t>
+  </si>
+  <si>
+    <t>max_quantity_preplan</t>
+  </si>
+  <si>
+    <t>max_quantity_period_1</t>
+  </si>
+  <si>
+    <t>max_quantity_period_2</t>
   </si>
 </sst>
 </file>
@@ -674,10 +701,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -685,46 +725,127 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="N1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
         <v>5000</v>
       </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2">
+        <v>2500</v>
+      </c>
+      <c r="D2">
+        <v>5000</v>
+      </c>
+      <c r="E2">
+        <v>5000</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>90</v>
+      </c>
+      <c r="J2">
+        <v>90</v>
+      </c>
+      <c r="K2">
+        <v>90</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
         <v>15</v>
       </c>
-      <c r="E2">
+      <c r="N2">
         <v>60.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3">
         <v>5000</v>
       </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3">
+        <v>1000</v>
+      </c>
+      <c r="D3">
+        <v>5000</v>
+      </c>
+      <c r="E3">
+        <v>5000</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>40</v>
+      </c>
+      <c r="J3">
+        <v>40</v>
+      </c>
+      <c r="K3">
+        <v>40</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>15</v>
       </c>
-      <c r="E3">
+      <c r="N3">
         <v>60.2</v>
       </c>
     </row>
@@ -736,17 +857,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" customWidth="1"/>
+    <col min="4" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="15.44140625" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -754,31 +878,49 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" t="s">
         <v>28</v>
       </c>
-      <c r="G1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="I1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" t="s">
+      <c r="P1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -786,31 +928,49 @@
         <v>20000</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>15000</v>
       </c>
       <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>60</v>
+      </c>
+      <c r="J2">
+        <v>60</v>
+      </c>
+      <c r="K2">
+        <v>60</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
         <v>14</v>
       </c>
-      <c r="H2">
+      <c r="N2">
         <v>25000</v>
       </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
         <v>58.4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -818,31 +978,49 @@
         <v>20000</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>15000</v>
       </c>
       <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>60</v>
+      </c>
+      <c r="J3">
+        <v>60</v>
+      </c>
+      <c r="K3">
+        <v>60</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>14</v>
       </c>
-      <c r="H3">
+      <c r="N3">
         <v>25000</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
         <v>58.1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -850,31 +1028,49 @@
         <v>20000</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>15000</v>
       </c>
       <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>60</v>
+      </c>
+      <c r="J4">
+        <v>60</v>
+      </c>
+      <c r="K4">
+        <v>60</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>14</v>
       </c>
-      <c r="H4">
+      <c r="N4">
         <v>25000</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
         <v>58.1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -882,31 +1078,49 @@
         <v>20000</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>15000</v>
       </c>
       <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>60</v>
+      </c>
+      <c r="J5">
+        <v>60</v>
+      </c>
+      <c r="K5">
+        <v>60</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>14</v>
       </c>
-      <c r="H5">
+      <c r="N5">
         <v>25000</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
         <v>58.2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -914,31 +1128,49 @@
         <v>20000</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>10000</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>15000</v>
       </c>
       <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>60</v>
+      </c>
+      <c r="J6">
+        <v>60</v>
+      </c>
+      <c r="K6">
+        <v>60</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>14</v>
       </c>
-      <c r="H6">
+      <c r="N6">
         <v>25000</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -946,27 +1178,45 @@
         <v>20000</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>10000</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>15000</v>
       </c>
       <c r="E7">
-        <v>2</v>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
+        <v>20000</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>60</v>
+      </c>
+      <c r="J7">
+        <v>60</v>
+      </c>
+      <c r="K7">
+        <v>60</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>14</v>
       </c>
-      <c r="H7">
+      <c r="N7">
         <v>25000</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
         <v>58.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented direct feed min and max ratios
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F239D22-8A54-415E-9A42-459279C0C526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860983D6-E12A-4E3F-86FD-346F1FCE1E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
   <si>
     <t>name</t>
   </si>
@@ -159,6 +159,24 @@
   </si>
   <si>
     <t>max_quantity_period_2</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_min_preplan</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_max_preplan</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_min_period_1</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_max_period_1</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_min_period_2</t>
+  </si>
+  <si>
+    <t>direct_feed_ratio_max_period_2</t>
   </si>
 </sst>
 </file>
@@ -622,21 +640,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="20.44140625" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="21.21875" customWidth="1"/>
+    <col min="10" max="10" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="21.21875" customWidth="1"/>
+    <col min="15" max="15" width="20.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -644,28 +665,46 @@
         <v>23</v>
       </c>
       <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>58</v>
       </c>
@@ -673,24 +712,42 @@
         <v>61</v>
       </c>
       <c r="C2">
+        <v>0.15</v>
+      </c>
+      <c r="D2">
+        <v>0.2</v>
+      </c>
+      <c r="E2">
         <v>3000</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>58</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>61</v>
       </c>
-      <c r="F2">
+      <c r="H2">
+        <v>0.15</v>
+      </c>
+      <c r="I2">
+        <v>0.2</v>
+      </c>
+      <c r="J2">
         <v>3000</v>
       </c>
-      <c r="G2">
+      <c r="K2">
         <v>58</v>
       </c>
-      <c r="H2">
+      <c r="L2">
         <v>61</v>
       </c>
-      <c r="I2">
+      <c r="M2">
+        <v>0.15</v>
+      </c>
+      <c r="N2">
+        <v>0.2</v>
+      </c>
+      <c r="O2">
         <v>3000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented blend options and user interaction to choose blend
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860983D6-E12A-4E3F-86FD-346F1FCE1E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C945E6C-6E44-4464-9915-D779C1912D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -712,10 +712,10 @@
         <v>61</v>
       </c>
       <c r="C2">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>3000</v>
@@ -727,10 +727,10 @@
         <v>61</v>
       </c>
       <c r="H2">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <v>3000</v>
@@ -742,10 +742,10 @@
         <v>61</v>
       </c>
       <c r="M2">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>3000</v>
@@ -826,7 +826,7 @@
         <v>5000</v>
       </c>
       <c r="C2">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="D2">
         <v>5000</v>
@@ -844,13 +844,13 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="J2">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="K2">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
@@ -870,7 +870,7 @@
         <v>5000</v>
       </c>
       <c r="C3">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="D3">
         <v>5000</v>
@@ -888,13 +888,13 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="L3" t="b">
         <v>1</v>
@@ -985,10 +985,10 @@
         <v>20000</v>
       </c>
       <c r="C2">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D2">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E2">
         <v>20000</v>
@@ -1018,7 +1018,7 @@
         <v>14</v>
       </c>
       <c r="N2">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1035,10 +1035,10 @@
         <v>20000</v>
       </c>
       <c r="C3">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D3">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E3">
         <v>20000</v>
@@ -1068,7 +1068,7 @@
         <v>14</v>
       </c>
       <c r="N3">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O3">
         <v>0</v>
@@ -1085,10 +1085,10 @@
         <v>20000</v>
       </c>
       <c r="C4">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D4">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E4">
         <v>20000</v>
@@ -1118,7 +1118,7 @@
         <v>14</v>
       </c>
       <c r="N4">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -1135,10 +1135,10 @@
         <v>20000</v>
       </c>
       <c r="C5">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D5">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E5">
         <v>20000</v>
@@ -1168,7 +1168,7 @@
         <v>14</v>
       </c>
       <c r="N5">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -1185,10 +1185,10 @@
         <v>20000</v>
       </c>
       <c r="C6">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D6">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E6">
         <v>20000</v>
@@ -1218,7 +1218,7 @@
         <v>14</v>
       </c>
       <c r="N6">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O6">
         <v>0</v>
@@ -1235,10 +1235,10 @@
         <v>20000</v>
       </c>
       <c r="C7">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="D7">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="E7">
         <v>20000</v>
@@ -1268,7 +1268,7 @@
         <v>14</v>
       </c>
       <c r="N7">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="O7">
         <v>0</v>

</xml_diff>

<commit_message>
Improved user interaction and reporting
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C945E6C-6E44-4464-9915-D779C1912D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D7E66A-C1DA-4BFD-A219-BA847E858B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -712,10 +712,10 @@
         <v>61</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="E2">
         <v>3000</v>
@@ -727,10 +727,10 @@
         <v>61</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="J2">
         <v>3000</v>
@@ -742,10 +742,10 @@
         <v>61</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="O2">
         <v>3000</v>
@@ -761,17 +761,17 @@
   <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.33203125" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -829,7 +829,7 @@
         <v>5000</v>
       </c>
       <c r="D2">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="E2">
         <v>5000</v>
@@ -844,13 +844,13 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
@@ -985,13 +985,13 @@
         <v>20000</v>
       </c>
       <c r="C2">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="D2">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="E2">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1153,13 +1153,13 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L5" t="b">
         <v>1</v>
@@ -1203,13 +1203,13 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L6" t="b">
         <v>1</v>
@@ -1253,13 +1253,13 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K7">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L7" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Improved user interactions (prompt user only when blend changes otherwise continue with the currently selected blend)
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/input/data.xlsx
+++ b/blendmaster_backend_OOP/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster_backend_OOP\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D7E66A-C1DA-4BFD-A219-BA847E858B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A3AAC4-14B8-41A7-8339-F30AD7AED835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15840" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -601,13 +601,13 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="F2">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="G2">
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -624,13 +624,13 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="F3">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="G3">
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -718,7 +718,7 @@
         <v>0.1</v>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="F2">
         <v>58</v>
@@ -733,7 +733,7 @@
         <v>0.1</v>
       </c>
       <c r="J2">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="K2">
         <v>58</v>
@@ -748,7 +748,7 @@
         <v>0.1</v>
       </c>
       <c r="O2">
-        <v>3000</v>
+        <v>3500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>